<commit_message>
Update DWH Mapping Excel
</commit_message>
<xml_diff>
--- a/Dokumentation/DWH_Mapping_Fakten_Dimensionen_v3.xlsx
+++ b/Dokumentation/DWH_Mapping_Fakten_Dimensionen_v3.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kaeseberg\Github\DVS\Dokumentation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{123846F9-5220-4465-A1B4-5C9BF47BF57C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{06D0C8DD-D6DF-49E4-AE2A-27F4D201C5D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1515,8 +1515,8 @@
   <cols>
     <col min="1" max="1" width="16" customWidth="1"/>
     <col min="2" max="2" width="31.265625" customWidth="1"/>
-    <col min="3" max="3" width="20" customWidth="1"/>
-    <col min="4" max="4" width="52" customWidth="1"/>
+    <col min="3" max="3" width="19.73046875" customWidth="1"/>
+    <col min="4" max="4" width="51.33203125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="26" customWidth="1"/>
     <col min="6" max="6" width="32" customWidth="1"/>
     <col min="7" max="7" width="44" customWidth="1"/>

</xml_diff>